<commit_message>
Versione pronta per report
</commit_message>
<xml_diff>
--- a/output/spreadsheets/MQT_device_selector_dataset_expected_fidelity.xlsx
+++ b/output/spreadsheets/MQT_device_selector_dataset_expected_fidelity.xlsx
@@ -208,70 +208,77 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DeviceSelectorDataset" displayName="DeviceSelectorDataset" ref="A1:BA5" headerRowCount="1">
-  <autoFilter ref="A1:BA5"/>
-  <tableColumns count="53">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DeviceSelectorDataset" displayName="DeviceSelectorDataset" ref="A1:BH9" headerRowCount="1">
+  <autoFilter ref="A1:BH9"/>
+  <tableColumns count="60">
     <tableColumn id="1" name="index"/>
     <tableColumn id="2" name="name"/>
     <tableColumn id="3" name="label_device"/>
-    <tableColumn id="4" name="score"/>
-    <tableColumn id="5" name="num_qubits"/>
-    <tableColumn id="6" name="depth"/>
-    <tableColumn id="7" name="program_communication"/>
-    <tableColumn id="8" name="critical_depth"/>
-    <tableColumn id="9" name="entanglement_ratio"/>
-    <tableColumn id="10" name="parallelism"/>
-    <tableColumn id="11" name="liveness"/>
-    <tableColumn id="12" name="gate_count_u3"/>
-    <tableColumn id="13" name="gate_count_u2"/>
-    <tableColumn id="14" name="gate_count_u1"/>
-    <tableColumn id="15" name="gate_count_cx"/>
-    <tableColumn id="16" name="gate_count_id"/>
-    <tableColumn id="17" name="gate_count_u0"/>
-    <tableColumn id="18" name="gate_count_u"/>
-    <tableColumn id="19" name="gate_count_p"/>
-    <tableColumn id="20" name="gate_count_x"/>
-    <tableColumn id="21" name="gate_count_y"/>
-    <tableColumn id="22" name="gate_count_z"/>
-    <tableColumn id="23" name="gate_count_h"/>
-    <tableColumn id="24" name="gate_count_s"/>
-    <tableColumn id="25" name="gate_count_sdg"/>
-    <tableColumn id="26" name="gate_count_t"/>
-    <tableColumn id="27" name="gate_count_tdg"/>
-    <tableColumn id="28" name="gate_count_rx"/>
-    <tableColumn id="29" name="gate_count_ry"/>
-    <tableColumn id="30" name="gate_count_rz"/>
-    <tableColumn id="31" name="gate_count_sx"/>
-    <tableColumn id="32" name="gate_count_sxdg"/>
-    <tableColumn id="33" name="gate_count_cz"/>
-    <tableColumn id="34" name="gate_count_cy"/>
-    <tableColumn id="35" name="gate_count_swap"/>
-    <tableColumn id="36" name="gate_count_ch"/>
-    <tableColumn id="37" name="gate_count_ccx"/>
-    <tableColumn id="38" name="gate_count_cswap"/>
-    <tableColumn id="39" name="gate_count_crx"/>
-    <tableColumn id="40" name="gate_count_cry"/>
-    <tableColumn id="41" name="gate_count_crz"/>
-    <tableColumn id="42" name="gate_count_cu1"/>
-    <tableColumn id="43" name="gate_count_cp"/>
-    <tableColumn id="44" name="gate_count_cu3"/>
-    <tableColumn id="45" name="gate_count_csx"/>
-    <tableColumn id="46" name="gate_count_cu"/>
-    <tableColumn id="47" name="gate_count_rxx"/>
-    <tableColumn id="48" name="gate_count_rzz"/>
-    <tableColumn id="49" name="gate_count_rccx"/>
-    <tableColumn id="50" name="gate_count_rc3x"/>
-    <tableColumn id="51" name="gate_count_c3x"/>
-    <tableColumn id="52" name="gate_count_c3sqrtx"/>
-    <tableColumn id="53" name="gate_count_c4x"/>
+    <tableColumn id="4" name="score_ibm_falcon_127"/>
+    <tableColumn id="5" name="score_quantinuum_h2_56"/>
+    <tableColumn id="6" name="qasm_found"/>
+    <tableColumn id="7" name="qasm_path"/>
+    <tableColumn id="8" name="source_num_qubits"/>
+    <tableColumn id="9" name="source_depth"/>
+    <tableColumn id="10" name="compiled_qasm_count"/>
+    <tableColumn id="11" name="compiled_qasm_devices"/>
+    <tableColumn id="12" name="num_qubits"/>
+    <tableColumn id="13" name="depth"/>
+    <tableColumn id="14" name="program_communication"/>
+    <tableColumn id="15" name="critical_depth"/>
+    <tableColumn id="16" name="entanglement_ratio"/>
+    <tableColumn id="17" name="parallelism"/>
+    <tableColumn id="18" name="liveness"/>
+    <tableColumn id="19" name="gate_count_u3"/>
+    <tableColumn id="20" name="gate_count_u2"/>
+    <tableColumn id="21" name="gate_count_u1"/>
+    <tableColumn id="22" name="gate_count_cx"/>
+    <tableColumn id="23" name="gate_count_id"/>
+    <tableColumn id="24" name="gate_count_u0"/>
+    <tableColumn id="25" name="gate_count_u"/>
+    <tableColumn id="26" name="gate_count_p"/>
+    <tableColumn id="27" name="gate_count_x"/>
+    <tableColumn id="28" name="gate_count_y"/>
+    <tableColumn id="29" name="gate_count_z"/>
+    <tableColumn id="30" name="gate_count_h"/>
+    <tableColumn id="31" name="gate_count_s"/>
+    <tableColumn id="32" name="gate_count_sdg"/>
+    <tableColumn id="33" name="gate_count_t"/>
+    <tableColumn id="34" name="gate_count_tdg"/>
+    <tableColumn id="35" name="gate_count_rx"/>
+    <tableColumn id="36" name="gate_count_ry"/>
+    <tableColumn id="37" name="gate_count_rz"/>
+    <tableColumn id="38" name="gate_count_sx"/>
+    <tableColumn id="39" name="gate_count_sxdg"/>
+    <tableColumn id="40" name="gate_count_cz"/>
+    <tableColumn id="41" name="gate_count_cy"/>
+    <tableColumn id="42" name="gate_count_swap"/>
+    <tableColumn id="43" name="gate_count_ch"/>
+    <tableColumn id="44" name="gate_count_ccx"/>
+    <tableColumn id="45" name="gate_count_cswap"/>
+    <tableColumn id="46" name="gate_count_crx"/>
+    <tableColumn id="47" name="gate_count_cry"/>
+    <tableColumn id="48" name="gate_count_crz"/>
+    <tableColumn id="49" name="gate_count_cu1"/>
+    <tableColumn id="50" name="gate_count_cp"/>
+    <tableColumn id="51" name="gate_count_cu3"/>
+    <tableColumn id="52" name="gate_count_csx"/>
+    <tableColumn id="53" name="gate_count_cu"/>
+    <tableColumn id="54" name="gate_count_rxx"/>
+    <tableColumn id="55" name="gate_count_rzz"/>
+    <tableColumn id="56" name="gate_count_rccx"/>
+    <tableColumn id="57" name="gate_count_rc3x"/>
+    <tableColumn id="58" name="gate_count_c3x"/>
+    <tableColumn id="59" name="gate_count_c3sqrtx"/>
+    <tableColumn id="60" name="gate_count_c4x"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="XMatrix" displayName="XMatrix" ref="A1:AX5" headerRowCount="1">
-  <autoFilter ref="A1:AX5"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="XMatrix" displayName="XMatrix" ref="A1:AX9" headerRowCount="1">
+  <autoFilter ref="A1:AX9"/>
   <tableColumns count="50">
     <tableColumn id="1" name="name"/>
     <tableColumn id="2" name="gate_count_u3"/>
@@ -667,7 +674,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4">
@@ -748,7 +755,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>In questo dataset locale c'e' un solo device candidato, quindi tutte le label sono quantinuum_h2_56.</t>
+          <t>In questo dataset locale ci sono 2 device candidati: ibm_falcon_127, quantinuum_h2_56.</t>
         </is>
       </c>
     </row>
@@ -760,7 +767,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>{"quantinuum_h2_56": 4}</t>
+          <t>{"ibm_falcon_127": 2, "quantinuum_h2_56": 6}</t>
         </is>
       </c>
     </row>
@@ -775,7 +782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA5"/>
+  <dimension ref="A1:BH9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -831,6 +838,13 @@
     <col width="14" customWidth="1" min="51" max="51"/>
     <col width="14" customWidth="1" min="52" max="52"/>
     <col width="14" customWidth="1" min="53" max="53"/>
+    <col width="14" customWidth="1" min="54" max="54"/>
+    <col width="14" customWidth="1" min="55" max="55"/>
+    <col width="14" customWidth="1" min="56" max="56"/>
+    <col width="14" customWidth="1" min="57" max="57"/>
+    <col width="14" customWidth="1" min="58" max="58"/>
+    <col width="14" customWidth="1" min="59" max="59"/>
+    <col width="14" customWidth="1" min="60" max="60"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -851,250 +865,285 @@
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>score</t>
+          <t>score_ibm_falcon_127</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
+          <t>score_quantinuum_h2_56</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>qasm_found</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>qasm_path</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>source_num_qubits</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>source_depth</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>compiled_qasm_count</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>compiled_qasm_devices</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
           <t>num_qubits</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="M1" s="4" t="inlineStr">
         <is>
           <t>depth</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="N1" s="4" t="inlineStr">
         <is>
           <t>program_communication</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="O1" s="4" t="inlineStr">
         <is>
           <t>critical_depth</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="P1" s="4" t="inlineStr">
         <is>
           <t>entanglement_ratio</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="Q1" s="4" t="inlineStr">
         <is>
           <t>parallelism</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="R1" s="4" t="inlineStr">
         <is>
           <t>liveness</t>
         </is>
       </c>
-      <c r="L1" s="4" t="inlineStr">
+      <c r="S1" s="4" t="inlineStr">
         <is>
           <t>gate_count_u3</t>
         </is>
       </c>
-      <c r="M1" s="4" t="inlineStr">
+      <c r="T1" s="4" t="inlineStr">
         <is>
           <t>gate_count_u2</t>
         </is>
       </c>
-      <c r="N1" s="4" t="inlineStr">
+      <c r="U1" s="4" t="inlineStr">
         <is>
           <t>gate_count_u1</t>
         </is>
       </c>
-      <c r="O1" s="4" t="inlineStr">
+      <c r="V1" s="4" t="inlineStr">
         <is>
           <t>gate_count_cx</t>
         </is>
       </c>
-      <c r="P1" s="4" t="inlineStr">
+      <c r="W1" s="4" t="inlineStr">
         <is>
           <t>gate_count_id</t>
         </is>
       </c>
-      <c r="Q1" s="4" t="inlineStr">
+      <c r="X1" s="4" t="inlineStr">
         <is>
           <t>gate_count_u0</t>
         </is>
       </c>
-      <c r="R1" s="4" t="inlineStr">
+      <c r="Y1" s="4" t="inlineStr">
         <is>
           <t>gate_count_u</t>
         </is>
       </c>
-      <c r="S1" s="4" t="inlineStr">
+      <c r="Z1" s="4" t="inlineStr">
         <is>
           <t>gate_count_p</t>
         </is>
       </c>
-      <c r="T1" s="4" t="inlineStr">
+      <c r="AA1" s="4" t="inlineStr">
         <is>
           <t>gate_count_x</t>
         </is>
       </c>
-      <c r="U1" s="4" t="inlineStr">
+      <c r="AB1" s="4" t="inlineStr">
         <is>
           <t>gate_count_y</t>
         </is>
       </c>
-      <c r="V1" s="4" t="inlineStr">
+      <c r="AC1" s="4" t="inlineStr">
         <is>
           <t>gate_count_z</t>
         </is>
       </c>
-      <c r="W1" s="4" t="inlineStr">
+      <c r="AD1" s="4" t="inlineStr">
         <is>
           <t>gate_count_h</t>
         </is>
       </c>
-      <c r="X1" s="4" t="inlineStr">
+      <c r="AE1" s="4" t="inlineStr">
         <is>
           <t>gate_count_s</t>
         </is>
       </c>
-      <c r="Y1" s="4" t="inlineStr">
+      <c r="AF1" s="4" t="inlineStr">
         <is>
           <t>gate_count_sdg</t>
         </is>
       </c>
-      <c r="Z1" s="4" t="inlineStr">
+      <c r="AG1" s="4" t="inlineStr">
         <is>
           <t>gate_count_t</t>
         </is>
       </c>
-      <c r="AA1" s="4" t="inlineStr">
+      <c r="AH1" s="4" t="inlineStr">
         <is>
           <t>gate_count_tdg</t>
         </is>
       </c>
-      <c r="AB1" s="4" t="inlineStr">
+      <c r="AI1" s="4" t="inlineStr">
         <is>
           <t>gate_count_rx</t>
         </is>
       </c>
-      <c r="AC1" s="4" t="inlineStr">
+      <c r="AJ1" s="4" t="inlineStr">
         <is>
           <t>gate_count_ry</t>
         </is>
       </c>
-      <c r="AD1" s="4" t="inlineStr">
+      <c r="AK1" s="4" t="inlineStr">
         <is>
           <t>gate_count_rz</t>
         </is>
       </c>
-      <c r="AE1" s="4" t="inlineStr">
+      <c r="AL1" s="4" t="inlineStr">
         <is>
           <t>gate_count_sx</t>
         </is>
       </c>
-      <c r="AF1" s="4" t="inlineStr">
+      <c r="AM1" s="4" t="inlineStr">
         <is>
           <t>gate_count_sxdg</t>
         </is>
       </c>
-      <c r="AG1" s="4" t="inlineStr">
+      <c r="AN1" s="4" t="inlineStr">
         <is>
           <t>gate_count_cz</t>
         </is>
       </c>
-      <c r="AH1" s="4" t="inlineStr">
+      <c r="AO1" s="4" t="inlineStr">
         <is>
           <t>gate_count_cy</t>
         </is>
       </c>
-      <c r="AI1" s="4" t="inlineStr">
+      <c r="AP1" s="4" t="inlineStr">
         <is>
           <t>gate_count_swap</t>
         </is>
       </c>
-      <c r="AJ1" s="4" t="inlineStr">
+      <c r="AQ1" s="4" t="inlineStr">
         <is>
           <t>gate_count_ch</t>
         </is>
       </c>
-      <c r="AK1" s="4" t="inlineStr">
+      <c r="AR1" s="4" t="inlineStr">
         <is>
           <t>gate_count_ccx</t>
         </is>
       </c>
-      <c r="AL1" s="4" t="inlineStr">
+      <c r="AS1" s="4" t="inlineStr">
         <is>
           <t>gate_count_cswap</t>
         </is>
       </c>
-      <c r="AM1" s="4" t="inlineStr">
+      <c r="AT1" s="4" t="inlineStr">
         <is>
           <t>gate_count_crx</t>
         </is>
       </c>
-      <c r="AN1" s="4" t="inlineStr">
+      <c r="AU1" s="4" t="inlineStr">
         <is>
           <t>gate_count_cry</t>
         </is>
       </c>
-      <c r="AO1" s="4" t="inlineStr">
+      <c r="AV1" s="4" t="inlineStr">
         <is>
           <t>gate_count_crz</t>
         </is>
       </c>
-      <c r="AP1" s="4" t="inlineStr">
+      <c r="AW1" s="4" t="inlineStr">
         <is>
           <t>gate_count_cu1</t>
         </is>
       </c>
-      <c r="AQ1" s="4" t="inlineStr">
+      <c r="AX1" s="4" t="inlineStr">
         <is>
           <t>gate_count_cp</t>
         </is>
       </c>
-      <c r="AR1" s="4" t="inlineStr">
+      <c r="AY1" s="4" t="inlineStr">
         <is>
           <t>gate_count_cu3</t>
         </is>
       </c>
-      <c r="AS1" s="4" t="inlineStr">
+      <c r="AZ1" s="4" t="inlineStr">
         <is>
           <t>gate_count_csx</t>
         </is>
       </c>
-      <c r="AT1" s="4" t="inlineStr">
+      <c r="BA1" s="4" t="inlineStr">
         <is>
           <t>gate_count_cu</t>
         </is>
       </c>
-      <c r="AU1" s="4" t="inlineStr">
+      <c r="BB1" s="4" t="inlineStr">
         <is>
           <t>gate_count_rxx</t>
         </is>
       </c>
-      <c r="AV1" s="4" t="inlineStr">
+      <c r="BC1" s="4" t="inlineStr">
         <is>
           <t>gate_count_rzz</t>
         </is>
       </c>
-      <c r="AW1" s="4" t="inlineStr">
+      <c r="BD1" s="4" t="inlineStr">
         <is>
           <t>gate_count_rccx</t>
         </is>
       </c>
-      <c r="AX1" s="4" t="inlineStr">
+      <c r="BE1" s="4" t="inlineStr">
         <is>
           <t>gate_count_rc3x</t>
         </is>
       </c>
-      <c r="AY1" s="4" t="inlineStr">
+      <c r="BF1" s="4" t="inlineStr">
         <is>
           <t>gate_count_c3x</t>
         </is>
       </c>
-      <c r="AZ1" s="4" t="inlineStr">
+      <c r="BG1" s="4" t="inlineStr">
         <is>
           <t>gate_count_c3sqrtx</t>
         </is>
       </c>
-      <c r="BA1" s="4" t="inlineStr">
+      <c r="BH1" s="4" t="inlineStr">
         <is>
           <t>gate_count_c4x</t>
         </is>
@@ -1106,73 +1155,77 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>qpeinexact_indep_qiskit_6</t>
+          <t>mini_wide_pair_28</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>quantinuum_h2_56</t>
+          <t>ibm_falcon_127</t>
         </is>
       </c>
       <c r="D2" s="6" t="n">
-        <v>0.9689400417</v>
-      </c>
-      <c r="E2" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="F2" s="7" t="n">
-        <v>17</v>
-      </c>
-      <c r="G2" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" s="8" t="n">
-        <v>0.7647058823529411</v>
-      </c>
-      <c r="I2" s="8" t="n">
-        <v>0.6071428571428571</v>
-      </c>
-      <c r="J2" s="8" t="n">
-        <v>0.1294117647058823</v>
-      </c>
-      <c r="K2" s="8" t="n">
-        <v>0.4901960784313725</v>
+        <v>0.9997664201000001</v>
+      </c>
+      <c r="E2" s="6" t="n">
+        <v>0.9982603852</v>
+      </c>
+      <c r="F2" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>mini-trainingset/uncompiled_circuit/mini_wide_pair_28.qasm</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="I2" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="J2" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>ibm_falcon_127, quantinuum_h2_56</t>
+        </is>
       </c>
       <c r="L2" s="7" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="M2" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="R2" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="N2" s="8" t="n">
+        <v>0.002645502645502645</v>
+      </c>
+      <c r="O2" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P2" s="8" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="Q2" s="8" t="n">
+        <v>0.01851851851851852</v>
+      </c>
+      <c r="R2" s="8" t="n">
+        <v>0.07142857142857142</v>
       </c>
       <c r="S2" s="7" t="n">
         <v>0</v>
       </c>
       <c r="T2" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U2" s="7" t="n">
         <v>0</v>
       </c>
       <c r="V2" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="X2" s="7" t="n">
         <v>0</v>
@@ -1193,7 +1246,7 @@
         <v>0</v>
       </c>
       <c r="AD2" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE2" s="7" t="n">
         <v>0</v>
@@ -1208,13 +1261,13 @@
         <v>0</v>
       </c>
       <c r="AI2" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AJ2" s="7" t="n">
         <v>0</v>
       </c>
       <c r="AK2" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AL2" s="7" t="n">
         <v>0</v>
@@ -1232,7 +1285,7 @@
         <v>0</v>
       </c>
       <c r="AQ2" s="7" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="AR2" s="7" t="n">
         <v>0</v>
@@ -1262,6 +1315,27 @@
         <v>0</v>
       </c>
       <c r="BA2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH2" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1271,7 +1345,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>twolocalrandom_indep_tket_4</t>
+          <t>mini_ring_5</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
@@ -1280,49 +1354,53 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>0.9639799053</v>
-      </c>
-      <c r="E3" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="F3" s="7" t="n">
-        <v>18</v>
-      </c>
-      <c r="G3" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="H3" s="8" t="n">
-        <v>0.7222222222222222</v>
-      </c>
-      <c r="I3" s="8" t="n">
-        <v>0.5294117647058824</v>
-      </c>
-      <c r="J3" s="8" t="n">
-        <v>0.2962962962962963</v>
-      </c>
-      <c r="K3" s="8" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.9794974601000001</v>
+      </c>
+      <c r="E3" s="6" t="n">
+        <v>0.991748589</v>
+      </c>
+      <c r="F3" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>mini-trainingset/uncompiled_circuit/mini_ring_5.qasm</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="I3" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="J3" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>ibm_falcon_127, quantinuum_h2_56</t>
+        </is>
       </c>
       <c r="L3" s="7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="M3" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O3" s="7" t="n">
-        <v>18</v>
-      </c>
-      <c r="P3" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q3" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="R3" s="7" t="n">
-        <v>0</v>
+        <v>7</v>
+      </c>
+      <c r="N3" s="8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="O3" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P3" s="8" t="n">
+        <v>0.7142857142857143</v>
+      </c>
+      <c r="Q3" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" s="8" t="n">
+        <v>0.3428571428571429</v>
       </c>
       <c r="S3" s="7" t="n">
         <v>0</v>
@@ -1334,7 +1412,7 @@
         <v>0</v>
       </c>
       <c r="V3" s="7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="W3" s="7" t="n">
         <v>0</v>
@@ -1355,10 +1433,10 @@
         <v>0</v>
       </c>
       <c r="AC3" s="7" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="AD3" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE3" s="7" t="n">
         <v>0</v>
@@ -1379,7 +1457,7 @@
         <v>0</v>
       </c>
       <c r="AK3" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AL3" s="7" t="n">
         <v>0</v>
@@ -1427,6 +1505,27 @@
         <v>0</v>
       </c>
       <c r="BA3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH3" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1436,7 +1535,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>qft_indep_qiskit_4</t>
+          <t>mini_parallel_4</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
@@ -1445,50 +1544,54 @@
         </is>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0.9842441682</v>
-      </c>
-      <c r="E4" s="7" t="n">
+        <v>0.9950525487</v>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>0.9965835907</v>
+      </c>
+      <c r="F4" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>mini-trainingset/uncompiled_circuit/mini_parallel_4.qasm</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="F4" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G4" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="H4" s="8" t="n">
+      <c r="I4" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="J4" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>ibm_falcon_127, quantinuum_h2_56</t>
+        </is>
+      </c>
+      <c r="L4" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="M4" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="N4" s="8" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="O4" s="8" t="n">
         <v>0.5</v>
       </c>
-      <c r="I4" s="8" t="n">
+      <c r="P4" s="8" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="Q4" s="8" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="R4" s="8" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="J4" s="8" t="n">
-        <v>0.1111111111111111</v>
-      </c>
-      <c r="K4" s="8" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="L4" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M4" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O4" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="R4" s="7" t="n">
-        <v>0</v>
-      </c>
       <c r="S4" s="7" t="n">
         <v>0</v>
       </c>
@@ -1499,10 +1602,10 @@
         <v>0</v>
       </c>
       <c r="V4" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W4" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="X4" s="7" t="n">
         <v>0</v>
@@ -1523,7 +1626,7 @@
         <v>0</v>
       </c>
       <c r="AD4" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AE4" s="7" t="n">
         <v>0</v>
@@ -1538,14 +1641,14 @@
         <v>0</v>
       </c>
       <c r="AI4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK4" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="AJ4" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK4" s="7" t="n">
-        <v>0</v>
-      </c>
       <c r="AL4" s="7" t="n">
         <v>0</v>
       </c>
@@ -1562,7 +1665,7 @@
         <v>0</v>
       </c>
       <c r="AQ4" s="7" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AR4" s="7" t="n">
         <v>0</v>
@@ -1592,6 +1695,27 @@
         <v>0</v>
       </c>
       <c r="BA4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH4" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1601,162 +1725,947 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>routing_indep_tket_2</t>
+          <t>mini_ghz_3</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
+          <t>ibm_falcon_127</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>0.9970911216</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>0.9966433884</v>
+      </c>
+      <c r="F5" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>mini-trainingset/uncompiled_circuit/mini_ghz_3.qasm</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="I5" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="J5" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>ibm_falcon_127, quantinuum_h2_56</t>
+        </is>
+      </c>
+      <c r="L5" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="M5" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="N5" s="8" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="O5" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P5" s="8" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="Q5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" s="8" t="n">
+        <v>0.5555555555555556</v>
+      </c>
+      <c r="S5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="V5" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="W5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH5" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>mini_bell_2</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
           <t>quantinuum_h2_56</t>
         </is>
       </c>
-      <c r="D5" s="6" t="n">
-        <v>0.9935960822</v>
-      </c>
-      <c r="E5" s="7" t="n">
+      <c r="D6" s="6" t="n">
+        <v>0.997817637</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>0.9982903339</v>
+      </c>
+      <c r="F6" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>mini-trainingset/uncompiled_circuit/mini_bell_2.qasm</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F5" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="G5" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="H5" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="I5" s="8" t="n">
-        <v>0.2727272727272727</v>
-      </c>
-      <c r="J5" s="8" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="K5" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="L5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" s="7" t="n">
+      <c r="I6" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="J6" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>ibm_falcon_127, quantinuum_h2_56</t>
+        </is>
+      </c>
+      <c r="L6" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="M6" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="N6" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="O6" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P6" s="8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Q6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" s="8" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="S6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="V6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="W6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH6" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>mini_single_3</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>quantinuum_h2_56</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>0.9998088771</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>0.9998800054</v>
+      </c>
+      <c r="F7" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>mini-trainingset/uncompiled_circuit/mini_single_3.qasm</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="P5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="R5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="S5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="T5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="U5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="V5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="W5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="X5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC5" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="AD5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA5" s="7" t="n">
+      <c r="I7" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="J7" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>ibm_falcon_127, quantinuum_h2_56</t>
+        </is>
+      </c>
+      <c r="L7" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="M7" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="N7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="R7" s="8" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="S7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="V7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="W7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH7" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>mini_chain_4</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>quantinuum_h2_56</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>0.9943350527</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>0.9950290109</v>
+      </c>
+      <c r="F8" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>mini-trainingset/uncompiled_circuit/mini_chain_4.qasm</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="I8" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="J8" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>ibm_falcon_127, quantinuum_h2_56</t>
+        </is>
+      </c>
+      <c r="L8" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="M8" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="N8" s="8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="O8" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P8" s="8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Q8" s="8" t="n">
+        <v>0.06666666666666665</v>
+      </c>
+      <c r="R8" s="8" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="S8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="V8" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="W8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA8" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD8" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK8" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH8" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>mini_wide_single_28</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>quantinuum_h2_56</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>0.9998147379</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>0.9998800054</v>
+      </c>
+      <c r="F9" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>mini-trainingset/uncompiled_circuit/mini_wide_single_28.qasm</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>ibm_falcon_127, quantinuum_h2_56</t>
+        </is>
+      </c>
+      <c r="L9" s="7" t="n">
+        <v>28</v>
+      </c>
+      <c r="M9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="8" t="n">
+        <v>0.07407407407407407</v>
+      </c>
+      <c r="R9" s="8" t="n">
+        <v>0.1071428571428571</v>
+      </c>
+      <c r="S9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="V9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="W9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH9" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1774,7 +2683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX5"/>
+  <dimension ref="A1:AX9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2084,7 +2993,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>qpeinexact_indep_qiskit_6</t>
+          <t>mini_wide_pair_28</t>
         </is>
       </c>
       <c r="B2" s="7" t="n">
@@ -2097,7 +3006,7 @@
         <v>0</v>
       </c>
       <c r="E2" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F2" s="7" t="n">
         <v>0</v>
@@ -2112,7 +3021,7 @@
         <v>0</v>
       </c>
       <c r="J2" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K2" s="7" t="n">
         <v>0</v>
@@ -2121,7 +3030,7 @@
         <v>0</v>
       </c>
       <c r="M2" s="7" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="N2" s="7" t="n">
         <v>0</v>
@@ -2142,7 +3051,7 @@
         <v>0</v>
       </c>
       <c r="T2" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U2" s="7" t="n">
         <v>0</v>
@@ -2157,88 +3066,88 @@
         <v>0</v>
       </c>
       <c r="Y2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR2" s="7" t="n">
+        <v>28</v>
+      </c>
+      <c r="AS2" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="Z2" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA2" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB2" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC2" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD2" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE2" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF2" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG2" s="7" t="n">
-        <v>15</v>
-      </c>
-      <c r="AH2" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI2" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ2" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK2" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL2" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM2" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN2" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO2" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP2" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ2" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR2" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="AS2" s="7" t="n">
-        <v>17</v>
-      </c>
       <c r="AT2" s="8" t="n">
-        <v>1</v>
+        <v>0.002645502645502645</v>
       </c>
       <c r="AU2" s="8" t="n">
-        <v>0.7647058823529411</v>
+        <v>1</v>
       </c>
       <c r="AV2" s="8" t="n">
-        <v>0.6071428571428571</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="AW2" s="8" t="n">
-        <v>0.1294117647058823</v>
+        <v>0.01851851851851852</v>
       </c>
       <c r="AX2" s="8" t="n">
-        <v>0.4901960784313725</v>
+        <v>0.07142857142857142</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>twolocalrandom_indep_tket_4</t>
+          <t>mini_ring_5</t>
         </is>
       </c>
       <c r="B3" s="7" t="n">
@@ -2251,7 +3160,7 @@
         <v>0</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="F3" s="7" t="n">
         <v>0</v>
@@ -2275,7 +3184,7 @@
         <v>0</v>
       </c>
       <c r="M3" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N3" s="7" t="n">
         <v>0</v>
@@ -2293,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="S3" s="7" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="T3" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U3" s="7" t="n">
         <v>0</v>
@@ -2368,31 +3277,31 @@
         <v>0</v>
       </c>
       <c r="AR3" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AS3" s="7" t="n">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="AT3" s="8" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="AU3" s="8" t="n">
-        <v>0.7222222222222222</v>
+        <v>1</v>
       </c>
       <c r="AV3" s="8" t="n">
-        <v>0.5294117647058824</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="AW3" s="8" t="n">
-        <v>0.2962962962962963</v>
+        <v>0</v>
       </c>
       <c r="AX3" s="8" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.3428571428571429</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>qft_indep_qiskit_4</t>
+          <t>mini_parallel_4</t>
         </is>
       </c>
       <c r="B4" s="7" t="n">
@@ -2405,7 +3314,7 @@
         <v>0</v>
       </c>
       <c r="E4" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F4" s="7" t="n">
         <v>0</v>
@@ -2429,7 +3338,7 @@
         <v>0</v>
       </c>
       <c r="M4" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N4" s="7" t="n">
         <v>0</v>
@@ -2450,7 +3359,7 @@
         <v>0</v>
       </c>
       <c r="T4" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U4" s="7" t="n">
         <v>0</v>
@@ -2465,7 +3374,7 @@
         <v>0</v>
       </c>
       <c r="Y4" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Z4" s="7" t="n">
         <v>0</v>
@@ -2489,7 +3398,7 @@
         <v>0</v>
       </c>
       <c r="AG4" s="7" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AH4" s="7" t="n">
         <v>0</v>
@@ -2525,19 +3434,19 @@
         <v>4</v>
       </c>
       <c r="AS4" s="7" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="AT4" s="8" t="n">
-        <v>1</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="AU4" s="8" t="n">
         <v>0.5</v>
       </c>
       <c r="AV4" s="8" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="AW4" s="8" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="AX4" s="8" t="n">
         <v>0.6666666666666666</v>
@@ -2546,7 +3455,7 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>routing_indep_tket_2</t>
+          <t>mini_ghz_3</t>
         </is>
       </c>
       <c r="B5" s="7" t="n">
@@ -2559,142 +3468,758 @@
         <v>0</v>
       </c>
       <c r="E5" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="V5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="W5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR5" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="F5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="R5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="S5" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="T5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="U5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="V5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="W5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="X5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR5" s="7" t="n">
+      <c r="AS5" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT5" s="8" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="AU5" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV5" s="8" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="AW5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX5" s="8" t="n">
+        <v>0.5555555555555556</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>mini_bell_2</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="V6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="W6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR6" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="AS5" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="AT5" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="AU5" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="AV5" s="8" t="n">
-        <v>0.2727272727272727</v>
-      </c>
-      <c r="AW5" s="8" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="AX5" s="8" t="n">
-        <v>1</v>
+      <c r="AS6" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT6" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU6" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV6" s="8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AW6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX6" s="8" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>mini_single_3</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="U7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="V7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="W7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR7" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="AS7" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW7" s="8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AX7" s="8" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>mini_chain_4</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="U8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="V8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="W8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR8" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="AS8" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="AT8" s="8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AU8" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV8" s="8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AW8" s="8" t="n">
+        <v>0.06666666666666665</v>
+      </c>
+      <c r="AX8" s="8" t="n">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>mini_wide_single_28</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="U9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="V9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="W9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR9" s="7" t="n">
+        <v>28</v>
+      </c>
+      <c r="AS9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW9" s="8" t="n">
+        <v>0.07407407407407407</v>
+      </c>
+      <c r="AX9" s="8" t="n">
+        <v>0.1071428571428571</v>
       </c>
     </row>
   </sheetData>

</xml_diff>